<commit_message>
update mit vollständigen Code
</commit_message>
<xml_diff>
--- a/System_Input.xlsx
+++ b/System_Input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avick\Documents\GitHub\Camper_Energiesysteme\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E2C6C7A-96CD-4C71-88BD-7EF874A3B115}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1424586C-F3A2-4610-85AB-E826BE2C59CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{51F61740-7428-4C3C-A169-54C94EF9AFFE}"/>
   </bookViews>
@@ -251,11 +251,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -591,65 +589,65 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF67F706-E5B8-4224-A49C-A5842118B29C}">
   <dimension ref="A1:BB5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.21875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="28.77734375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="29.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="26.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="31.109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="26.21875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="31" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="30" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="31.21875" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="28.77734375" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="26.77734375" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="34" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="26.21875" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="31" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="28.44140625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="28.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -719,73 +717,73 @@
       <c r="W1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="Z1" t="s">
         <v>42</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AA1" t="s">
         <v>24</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AB1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AC1" t="s">
         <v>26</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AD1" t="s">
         <v>27</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AE1" t="s">
         <v>43</v>
       </c>
       <c r="AF1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AG1" t="s">
         <v>29</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AH1" t="s">
         <v>30</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AI1" t="s">
         <v>44</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AJ1" t="s">
         <v>31</v>
       </c>
       <c r="AK1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AL1" t="s">
         <v>33</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AM1" t="s">
         <v>34</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AN1" t="s">
         <v>45</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AO1" t="s">
         <v>35</v>
       </c>
       <c r="AP1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AQ1" t="s">
         <v>46</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AR1" t="s">
         <v>47</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AS1" t="s">
         <v>48</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AT1" t="s">
         <v>49</v>
       </c>
       <c r="AU1" t="s">
@@ -797,23 +795,23 @@
       <c r="AW1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="AX1" s="2" t="s">
+      <c r="AX1" t="s">
         <v>53</v>
       </c>
-      <c r="AY1" s="2" t="s">
+      <c r="AY1" t="s">
         <v>56</v>
       </c>
-      <c r="AZ1" s="2" t="s">
+      <c r="AZ1" t="s">
         <v>52</v>
       </c>
-      <c r="BA1" s="2" t="s">
+      <c r="BA1" t="s">
         <v>54</v>
       </c>
       <c r="BB1" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:54" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -913,7 +911,7 @@
       <c r="AW2" s="1"/>
       <c r="BB2" s="1"/>
     </row>
-    <row r="3" spans="1:54" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1013,7 +1011,7 @@
       <c r="AW3" s="1"/>
       <c r="BB3" s="1"/>
     </row>
-    <row r="4" spans="1:54" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -1113,7 +1111,7 @@
       <c r="AW4" s="1"/>
       <c r="BB4" s="1"/>
     </row>
-    <row r="5" spans="1:54" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>

</xml_diff>